<commit_message>
I have written the python code to add all the modules into my database using the csv files that I created through R
</commit_message>
<xml_diff>
--- a/Faculties/Law/Postgrad Law.xlsx
+++ b/Faculties/Law/Postgrad Law.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d24d4a286855a075/Desktop/Team_6_repo/Team19/Faculties/Law/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mwamb\OneDrive\Desktop\Team_6_repo\Team19\Faculties\Law\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="11_F25DC773A252ABDACC10480281DB6CA25BDE58F3" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7ABB1A20-5A92-4CA3-A979-05DC5261319D}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE97DF15-7A78-4130-A7C6-9EB71B3AEB7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12048" yWindow="3312" windowWidth="9984" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="13776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="396" uniqueCount="175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="396" uniqueCount="176">
   <si>
     <t>Module Code</t>
   </si>
@@ -186,9 +186,6 @@
     <t>Anti-Corruption Law 811</t>
   </si>
   <si>
-    <t>LLM</t>
-  </si>
-  <si>
     <t>AML811</t>
   </si>
   <si>
@@ -201,9 +198,6 @@
     <t>Comparative Constitutional Law 811</t>
   </si>
   <si>
-    <t>LLM, MPhil</t>
-  </si>
-  <si>
     <t>CDS811</t>
   </si>
   <si>
@@ -528,28 +522,37 @@
     <t>Research Paper 805 / 806</t>
   </si>
   <si>
-    <t xml:space="preserve">PGDip  Public Law </t>
-  </si>
-  <si>
-    <t xml:space="preserve">PGDip  Environmental Law &amp; Management </t>
-  </si>
-  <si>
-    <t xml:space="preserve">PGDip  Fintech Law &amp; Regulation </t>
-  </si>
-  <si>
-    <t xml:space="preserve">PGDip  Labour Law </t>
-  </si>
-  <si>
-    <t xml:space="preserve">PGDip  Tax Law </t>
-  </si>
-  <si>
-    <t xml:space="preserve">LLM, MPhil, LLM  LPFL </t>
-  </si>
-  <si>
-    <t xml:space="preserve">LLM  7811 </t>
-  </si>
-  <si>
-    <t xml:space="preserve">LLM  LPFL </t>
+    <t xml:space="preserve">PGDip Environmental Law and Management 7712 </t>
+  </si>
+  <si>
+    <t>PGDip Fintech Law and Regulation 7702</t>
+  </si>
+  <si>
+    <t>PGDip Public Law 7711</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PGDip Fintech Law and Regulation 7702 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">PGDip Labour Law 7701 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">PGDip Tax Law 7721 </t>
+  </si>
+  <si>
+    <t>LLM 7801, LLM 7821, LLM 7822</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LLM 7801, LLM 7821, LLM 7822 7811 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">LLM 7801, LLM 7821, LLM 7822 LPFL </t>
+  </si>
+  <si>
+    <t>LLM 7801, LLM 7821, LLM 7822, MPhil 7871, MPhil 7860, MPhil 7861</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LLM 7801, LLM 7821, LLM 7822, MPhil 7871, MPhil 7860, MPhil 7861, LLM 7801, LLM 7821, LLM 7822 LPFL </t>
   </si>
 </sst>
 </file>
@@ -886,6 +889,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F79"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="4" max="4" width="26.21875" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
@@ -967,7 +973,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>13</v>
       </c>
@@ -978,7 +984,7 @@
         <v>1</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>8</v>
@@ -998,7 +1004,7 @@
         <v>1</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>8</v>
@@ -1018,7 +1024,7 @@
         <v>1</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>8</v>
@@ -1038,7 +1044,7 @@
         <v>1</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>8</v>
@@ -1047,7 +1053,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="72" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>21</v>
       </c>
@@ -1058,7 +1064,7 @@
         <v>1</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>8</v>
@@ -1078,7 +1084,7 @@
         <v>1</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>8</v>
@@ -1098,7 +1104,7 @@
         <v>1</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>8</v>
@@ -1118,7 +1124,7 @@
         <v>1</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>8</v>
@@ -1178,7 +1184,7 @@
         <v>1</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>8</v>
@@ -1198,7 +1204,7 @@
         <v>1</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E16" s="1" t="s">
         <v>8</v>
@@ -1218,7 +1224,7 @@
         <v>1</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E17" s="1" t="s">
         <v>8</v>
@@ -1238,7 +1244,7 @@
         <v>1</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="E18" s="1" t="s">
         <v>8</v>
@@ -1278,7 +1284,7 @@
         <v>1</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="E20" s="1" t="s">
         <v>8</v>
@@ -1298,7 +1304,7 @@
         <v>1</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="E21" s="1" t="s">
         <v>8</v>
@@ -1318,7 +1324,7 @@
         <v>1</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="E22" s="1" t="s">
         <v>8</v>
@@ -1338,7 +1344,7 @@
         <v>1</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="E23" s="1" t="s">
         <v>8</v>
@@ -1358,7 +1364,7 @@
         <v>1</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>53</v>
+        <v>171</v>
       </c>
       <c r="E24" s="1" t="s">
         <v>8</v>
@@ -1369,16 +1375,16 @@
     </row>
     <row r="25" spans="1:6" ht="72" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B25" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="B25" s="1" t="s">
-        <v>55</v>
-      </c>
       <c r="C25" s="1">
         <v>1</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>53</v>
+        <v>171</v>
       </c>
       <c r="E25" s="1" t="s">
         <v>8</v>
@@ -1389,16 +1395,16 @@
     </row>
     <row r="26" spans="1:6" ht="72" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B26" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="B26" s="1" t="s">
-        <v>57</v>
-      </c>
       <c r="C26" s="1">
         <v>1</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>58</v>
+        <v>174</v>
       </c>
       <c r="E26" s="1" t="s">
         <v>8</v>
@@ -1409,16 +1415,16 @@
     </row>
     <row r="27" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C27" s="1">
         <v>1</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>58</v>
+        <v>174</v>
       </c>
       <c r="E27" s="1" t="s">
         <v>8</v>
@@ -1429,16 +1435,16 @@
     </row>
     <row r="28" spans="1:6" ht="72" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C28" s="1">
         <v>1</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>58</v>
+        <v>174</v>
       </c>
       <c r="E28" s="1" t="s">
         <v>8</v>
@@ -1449,16 +1455,16 @@
     </row>
     <row r="29" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C29" s="1">
         <v>1</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>58</v>
+        <v>174</v>
       </c>
       <c r="E29" s="1" t="s">
         <v>8</v>
@@ -1469,16 +1475,16 @@
     </row>
     <row r="30" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C30" s="1">
         <v>1</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>53</v>
+        <v>171</v>
       </c>
       <c r="E30" s="1" t="s">
         <v>8</v>
@@ -1489,16 +1495,16 @@
     </row>
     <row r="31" spans="1:6" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C31" s="1">
         <v>1</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>53</v>
+        <v>171</v>
       </c>
       <c r="E31" s="1" t="s">
         <v>8</v>
@@ -1509,16 +1515,16 @@
     </row>
     <row r="32" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C32" s="1">
         <v>1</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>53</v>
+        <v>171</v>
       </c>
       <c r="E32" s="1" t="s">
         <v>8</v>
@@ -1529,16 +1535,16 @@
     </row>
     <row r="33" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C33" s="1">
         <v>1</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>58</v>
+        <v>174</v>
       </c>
       <c r="E33" s="1" t="s">
         <v>8</v>
@@ -1549,16 +1555,16 @@
     </row>
     <row r="34" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C34" s="1">
         <v>1</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="E34" s="1" t="s">
         <v>8</v>
@@ -1569,16 +1575,16 @@
     </row>
     <row r="35" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C35" s="1">
         <v>1</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="E35" s="1" t="s">
         <v>8</v>
@@ -1589,19 +1595,19 @@
     </row>
     <row r="36" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C36" s="1">
+        <v>1</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="E36" s="1" t="s">
         <v>77</v>
-      </c>
-      <c r="B36" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="C36" s="1">
-        <v>1</v>
-      </c>
-      <c r="D36" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="E36" s="1" t="s">
-        <v>79</v>
       </c>
       <c r="F36" s="1" t="s">
         <v>8</v>
@@ -1609,16 +1615,16 @@
     </row>
     <row r="37" spans="1:6" ht="72" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C37" s="1">
         <v>1</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>58</v>
+        <v>174</v>
       </c>
       <c r="E37" s="1" t="s">
         <v>8</v>
@@ -1629,19 +1635,19 @@
     </row>
     <row r="38" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C38" s="1">
         <v>1</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>53</v>
+        <v>171</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F38" s="1" t="s">
         <v>8</v>
@@ -1649,16 +1655,16 @@
     </row>
     <row r="39" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C39" s="1">
         <v>1</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>58</v>
+        <v>174</v>
       </c>
       <c r="E39" s="1" t="s">
         <v>8</v>
@@ -1669,16 +1675,16 @@
     </row>
     <row r="40" spans="1:6" ht="72" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C40" s="1">
         <v>1</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>58</v>
+        <v>174</v>
       </c>
       <c r="E40" s="1" t="s">
         <v>8</v>
@@ -1689,16 +1695,16 @@
     </row>
     <row r="41" spans="1:6" ht="72" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C41" s="1">
         <v>1</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>58</v>
+        <v>174</v>
       </c>
       <c r="E41" s="1" t="s">
         <v>8</v>
@@ -1709,16 +1715,16 @@
     </row>
     <row r="42" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C42" s="1">
         <v>1</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>53</v>
+        <v>171</v>
       </c>
       <c r="E42" s="1" t="s">
         <v>8</v>
@@ -1729,16 +1735,16 @@
     </row>
     <row r="43" spans="1:6" ht="72" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C43" s="1">
         <v>1</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>53</v>
+        <v>171</v>
       </c>
       <c r="E43" s="1" t="s">
         <v>8</v>
@@ -1749,16 +1755,16 @@
     </row>
     <row r="44" spans="1:6" ht="72" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C44" s="1">
         <v>1</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>58</v>
+        <v>174</v>
       </c>
       <c r="E44" s="1" t="s">
         <v>8</v>
@@ -1769,16 +1775,16 @@
     </row>
     <row r="45" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C45" s="1">
         <v>1</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>58</v>
+        <v>174</v>
       </c>
       <c r="E45" s="1" t="s">
         <v>8</v>
@@ -1789,16 +1795,16 @@
     </row>
     <row r="46" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C46" s="1">
         <v>1</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>58</v>
+        <v>174</v>
       </c>
       <c r="E46" s="1" t="s">
         <v>8</v>
@@ -1809,16 +1815,16 @@
     </row>
     <row r="47" spans="1:6" ht="72" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C47" s="1">
         <v>1</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>58</v>
+        <v>174</v>
       </c>
       <c r="E47" s="1" t="s">
         <v>8</v>
@@ -1829,16 +1835,16 @@
     </row>
     <row r="48" spans="1:6" ht="72" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="C48" s="1">
         <v>1</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>58</v>
+        <v>174</v>
       </c>
       <c r="E48" s="1" t="s">
         <v>8</v>
@@ -1849,16 +1855,16 @@
     </row>
     <row r="49" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C49" s="1">
         <v>1</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>58</v>
+        <v>174</v>
       </c>
       <c r="E49" s="1" t="s">
         <v>8</v>
@@ -1869,16 +1875,16 @@
     </row>
     <row r="50" spans="1:6" ht="72" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C50" s="1">
         <v>1</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>58</v>
+        <v>174</v>
       </c>
       <c r="E50" s="1" t="s">
         <v>8</v>
@@ -1889,36 +1895,36 @@
     </row>
     <row r="51" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A51" s="2" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C51" s="1">
         <v>1</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="E51" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F51" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="52" spans="1:6" ht="72" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="C52" s="1">
         <v>1</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>58</v>
+        <v>174</v>
       </c>
       <c r="E52" s="1" t="s">
         <v>8</v>
@@ -1929,56 +1935,56 @@
     </row>
     <row r="53" spans="1:6" ht="72" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="B53" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="C53" s="1">
+        <v>1</v>
+      </c>
+      <c r="D53" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="E53" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F53" s="1" t="s">
         <v>112</v>
-      </c>
-      <c r="B53" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="C53" s="1">
-        <v>1</v>
-      </c>
-      <c r="D53" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="E53" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F53" s="1" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="54" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="C54" s="1">
         <v>1</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>58</v>
+        <v>174</v>
       </c>
       <c r="E54" s="1" t="s">
         <v>8</v>
       </c>
       <c r="F54" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
     </row>
     <row r="55" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="C55" s="1">
         <v>1</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>58</v>
+        <v>174</v>
       </c>
       <c r="E55" s="1" t="s">
         <v>8</v>
@@ -1989,16 +1995,16 @@
     </row>
     <row r="56" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A56" s="2" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C56" s="1">
         <v>1</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>58</v>
+        <v>174</v>
       </c>
       <c r="E56" s="1" t="s">
         <v>8</v>
@@ -2009,16 +2015,16 @@
     </row>
     <row r="57" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A57" s="2" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="C57" s="1">
         <v>1</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>58</v>
+        <v>174</v>
       </c>
       <c r="E57" s="1" t="s">
         <v>8</v>
@@ -2029,16 +2035,16 @@
     </row>
     <row r="58" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A58" s="2" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="C58" s="1">
         <v>1</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="E58" s="1" t="s">
         <v>8</v>
@@ -2049,16 +2055,16 @@
     </row>
     <row r="59" spans="1:6" ht="72" x14ac:dyDescent="0.3">
       <c r="A59" s="2" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C59" s="1">
         <v>1</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>58</v>
+        <v>174</v>
       </c>
       <c r="E59" s="1" t="s">
         <v>8</v>
@@ -2069,16 +2075,16 @@
     </row>
     <row r="60" spans="1:6" ht="72" x14ac:dyDescent="0.3">
       <c r="A60" s="2" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="C60" s="1">
         <v>1</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>58</v>
+        <v>174</v>
       </c>
       <c r="E60" s="1" t="s">
         <v>8</v>
@@ -2089,16 +2095,16 @@
     </row>
     <row r="61" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A61" s="2" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="C61" s="1">
         <v>1</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>58</v>
+        <v>174</v>
       </c>
       <c r="E61" s="1" t="s">
         <v>8</v>
@@ -2109,16 +2115,16 @@
     </row>
     <row r="62" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A62" s="2" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C62" s="1">
         <v>1</v>
       </c>
       <c r="D62" s="1" t="s">
-        <v>58</v>
+        <v>174</v>
       </c>
       <c r="E62" s="1" t="s">
         <v>8</v>
@@ -2129,16 +2135,16 @@
     </row>
     <row r="63" spans="1:6" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A63" s="2" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="C63" s="1">
         <v>1</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="E63" s="1" t="s">
         <v>8</v>
@@ -2149,16 +2155,16 @@
     </row>
     <row r="64" spans="1:6" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A64" s="2" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C64" s="1">
         <v>1</v>
       </c>
       <c r="D64" s="1" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="E64" s="1" t="s">
         <v>8</v>
@@ -2169,16 +2175,16 @@
     </row>
     <row r="65" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A65" s="2" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="C65" s="1">
         <v>1</v>
       </c>
       <c r="D65" s="1" t="s">
-        <v>58</v>
+        <v>174</v>
       </c>
       <c r="E65" s="1" t="s">
         <v>8</v>
@@ -2189,16 +2195,16 @@
     </row>
     <row r="66" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A66" s="2" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="C66" s="1">
         <v>1</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>58</v>
+        <v>174</v>
       </c>
       <c r="E66" s="1" t="s">
         <v>8</v>
@@ -2209,16 +2215,16 @@
     </row>
     <row r="67" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A67" s="2" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="C67" s="1">
         <v>1</v>
       </c>
       <c r="D67" s="1" t="s">
-        <v>58</v>
+        <v>174</v>
       </c>
       <c r="E67" s="1" t="s">
         <v>8</v>
@@ -2229,16 +2235,16 @@
     </row>
     <row r="68" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A68" s="2" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="C68" s="1">
         <v>1</v>
       </c>
       <c r="D68" s="1" t="s">
-        <v>58</v>
+        <v>174</v>
       </c>
       <c r="E68" s="1" t="s">
         <v>8</v>
@@ -2249,16 +2255,16 @@
     </row>
     <row r="69" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A69" s="2" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="C69" s="1">
         <v>1</v>
       </c>
       <c r="D69" s="1" t="s">
-        <v>58</v>
+        <v>174</v>
       </c>
       <c r="E69" s="1" t="s">
         <v>8</v>
@@ -2269,16 +2275,16 @@
     </row>
     <row r="70" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A70" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="C70" s="1">
         <v>1</v>
       </c>
       <c r="D70" s="1" t="s">
-        <v>53</v>
+        <v>171</v>
       </c>
       <c r="E70" s="1" t="s">
         <v>8</v>
@@ -2289,16 +2295,16 @@
     </row>
     <row r="71" spans="1:6" ht="72" x14ac:dyDescent="0.3">
       <c r="A71" s="2" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="C71" s="1">
         <v>1</v>
       </c>
       <c r="D71" s="1" t="s">
-        <v>58</v>
+        <v>174</v>
       </c>
       <c r="E71" s="1" t="s">
         <v>8</v>
@@ -2309,16 +2315,16 @@
     </row>
     <row r="72" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A72" s="2" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="C72" s="1">
         <v>1</v>
       </c>
       <c r="D72" s="1" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="E72" s="1" t="s">
         <v>8</v>
@@ -2329,16 +2335,16 @@
     </row>
     <row r="73" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A73" s="2" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="C73" s="1">
         <v>1</v>
       </c>
       <c r="D73" s="1" t="s">
-        <v>58</v>
+        <v>174</v>
       </c>
       <c r="E73" s="1" t="s">
         <v>8</v>
@@ -2349,16 +2355,16 @@
     </row>
     <row r="74" spans="1:6" ht="72" x14ac:dyDescent="0.3">
       <c r="A74" s="2" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="C74" s="1">
         <v>1</v>
       </c>
       <c r="D74" s="1" t="s">
-        <v>58</v>
+        <v>174</v>
       </c>
       <c r="E74" s="1" t="s">
         <v>8</v>
@@ -2369,16 +2375,16 @@
     </row>
     <row r="75" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A75" s="2" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="C75" s="1">
         <v>1</v>
       </c>
       <c r="D75" s="1" t="s">
-        <v>53</v>
+        <v>171</v>
       </c>
       <c r="E75" s="1" t="s">
         <v>8</v>
@@ -2389,16 +2395,16 @@
     </row>
     <row r="76" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A76" s="2" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="C76" s="3">
         <v>46024</v>
       </c>
       <c r="D76" s="1" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="E76" s="1" t="s">
         <v>8</v>
@@ -2409,16 +2415,16 @@
     </row>
     <row r="77" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A77" s="2" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="C77" s="3">
         <v>46024</v>
       </c>
       <c r="D77" s="1" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="E77" s="1" t="s">
         <v>8</v>
@@ -2429,16 +2435,16 @@
     </row>
     <row r="78" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A78" s="2" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="C78" s="3">
         <v>46024</v>
       </c>
       <c r="D78" s="1" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="E78" s="1" t="s">
         <v>8</v>
@@ -2449,16 +2455,16 @@
     </row>
     <row r="79" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A79" s="2" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="C79" s="3">
         <v>46024</v>
       </c>
       <c r="D79" s="1" t="s">
-        <v>58</v>
+        <v>174</v>
       </c>
       <c r="E79" s="1" t="s">
         <v>8</v>

</xml_diff>

<commit_message>
I have solved the in review AI feature, I just need to now solve the main AI review page
</commit_message>
<xml_diff>
--- a/Faculties/Law/Postgrad Law.xlsx
+++ b/Faculties/Law/Postgrad Law.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mwamb\OneDrive\Desktop\Team_6_repo\Team19\Faculties\Law\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d24d4a286855a075/Desktop/Team_6_repo/Team19/Faculties/Law/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE97DF15-7A78-4130-A7C6-9EB71B3AEB7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="13_ncr:1_{BE97DF15-7A78-4130-A7C6-9EB71B3AEB7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C38FC5E7-1F0E-48D2-9B36-0D4E7E66973C}"/>
   <bookViews>
     <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="13776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="396" uniqueCount="176">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="555" uniqueCount="328">
   <si>
     <t>Module Code</t>
   </si>
@@ -553,13 +553,565 @@
   </si>
   <si>
     <t xml:space="preserve">LLM 7801, LLM 7821, LLM 7822, MPhil 7871, MPhil 7860, MPhil 7861, LLM 7801, LLM 7821, LLM 7822 LPFL </t>
+  </si>
+  <si>
+    <t>Learning Outcome</t>
+  </si>
+  <si>
+    <t>Credits</t>
+  </si>
+  <si>
+    <t>Main Content</t>
+  </si>
+  <si>
+    <t>Discuss the main principles of administrative law; evaluate administrative powers and jurisdiction; analyze administrative action as per PAJA; and apply requirements for valid administrative actions to practical scenarios.</t>
+  </si>
+  <si>
+    <t>Foundations of administrative law; PAJA; powers and jurisdiction; action and control; valid administrative action requirements; standing and procedure; and remedies.</t>
+  </si>
+  <si>
+    <t>Articulate values underlying the Constitution and evaluate its principles; interpret the Constitution in hypothetical scenarios; evaluate government structure and powers; and compare the SA constitution within international contexts.</t>
+  </si>
+  <si>
+    <t>Constitutional values and principles; constitutional history; constitutional interpretation; Bill of Rights; federalism; and the separation of powers.</t>
+  </si>
+  <si>
+    <t>Critically evaluate the intersection between criminal justice systems and human rights in Africa, specifically focusing on vulnerable groups and unusual circumstances (e.g., states of emergency and disaster).</t>
+  </si>
+  <si>
+    <t>Criminal justice systems and human rights in Africa.</t>
+  </si>
+  <si>
+    <t>Identify and critically discuss the main rules, procedures, and principles of South African Environmental Law.</t>
+  </si>
+  <si>
+    <t>South African Environmental Law.</t>
+  </si>
+  <si>
+    <t>Critically discuss the nature, scope, and function of environmental governance; analyze rules, theories, and foundations in SA; and evaluate the Constitution and enabling legal framework.</t>
+  </si>
+  <si>
+    <t>Environmental governance in South Africa.</t>
+  </si>
+  <si>
+    <t>Critically discuss and apply Administrative Law principles to Environmental Law; evaluate administrative powers/jurisdiction; and analyze just administrative action.</t>
+  </si>
+  <si>
+    <t>Foundations and rules of Administrative Law in environmental context; Constitution (environmental right, access to info); requirements for valid action; and remedies.</t>
+  </si>
+  <si>
+    <t>Critically discuss principles of environmental management and their link to governance; discuss integrated management; and evaluate the rationale behind Environmental Impact Assessments.</t>
+  </si>
+  <si>
+    <t>Environmental Impact Assessment and general environmental management.</t>
+  </si>
+  <si>
+    <r>
+      <t>Consult the Centre for African Fintech, Innovation and Law (CAFIL) for detailed outcomes</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>Introduction to concepts in Fintech Law.</t>
+  </si>
+  <si>
+    <t>Banking system; virtual currencies, cryptocurrencies, and central bank digital currencies; and mobile money/financial inclusion.</t>
+  </si>
+  <si>
+    <t>Distinguish between payment systems regulation and oversight; and critically discuss and evaluate the meaning and legal nature of fintech payments.</t>
+  </si>
+  <si>
+    <t>Fintech payment regulation.</t>
+  </si>
+  <si>
+    <t>Critically discuss the meaning and nature of financial inclusion and integrity; and analyze their relationship with Fintech.</t>
+  </si>
+  <si>
+    <t>Trade-offs in Fintech regulation.</t>
+  </si>
+  <si>
+    <t>Evaluate the constitution and enabling framework for multi-level government in SA; locate the system within international debates; and compare provincial government finance sources.</t>
+  </si>
+  <si>
+    <t>Power distribution between national, provincial, and local government; constitutional framework; multi-level finance; and intergovernmental relations.</t>
+  </si>
+  <si>
+    <t>Articulate the constitution and enabling framework for local government in SA; identify strategies to integrate ethics and good governance; and locate the system within international debates.</t>
+  </si>
+  <si>
+    <t>Local government.</t>
+  </si>
+  <si>
+    <t>Critically analyze the elements of collective bargaining (including industrial action); demonstrate ability to engage with practical requirements; and apply statutory provisions for business transfers.</t>
+  </si>
+  <si>
+    <t>Historical development of SA labour law; contract principles; the constitutional framework (LRA, BCEA, EEA); legal interpretation; and collective bargaining.</t>
+  </si>
+  <si>
+    <t>Analyze concepts relevant to dismissal and unfair labour practices; demonstrate knowledge of constitutional/international rights; explain the role of common law; and apply SA labour legislation.</t>
+  </si>
+  <si>
+    <t>The right to fair labour practices.</t>
+  </si>
+  <si>
+    <r>
+      <t>Consult the Mercantile and Labour Law Department for detailed outcomes</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>Labour dispute resolution.</t>
+  </si>
+  <si>
+    <t>Demonstrate an understanding of ethical issues in conciliation and arbitration; explain and apply conciliation process elements; and demonstrate ability to conduct conciliation.</t>
+  </si>
+  <si>
+    <t>Conciliation; con-arb; conducting arbitration; representation; duties and powers; evidence admissibility; and arbitration awards (variation, rescission, and review).</t>
+  </si>
+  <si>
+    <r>
+      <t>Consult the Dullah Omar Institute for detailed outcomes</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>Detention and oversight, with specific reference to vulnerable groups and emergency/disaster situations.</t>
+  </si>
+  <si>
+    <t>Critically analyze "gross income" and constituent elements; understand residence and "place of effective management"; interpret source rules; and solve problems in factual scenarios.</t>
+  </si>
+  <si>
+    <t>Interpretation of fiscal statutes; Constitution impact; gross income (resident/non-resident); partnerships; revenue vs capital; and taxation of cryptocurrency.</t>
+  </si>
+  <si>
+    <t>Critically analyze fundamental concepts in international taxation; understand OECD model conventions; interpret double tax agreements; and evaluate international transactions.</t>
+  </si>
+  <si>
+    <t>International tax law.</t>
+  </si>
+  <si>
+    <t>Analyze legal concepts under the TAA, PAJA, and the Constitution; explain taxpayer rights (privacy, property, access); and interpret rules governing appeals and objections.</t>
+  </si>
+  <si>
+    <t>Inter-relationship between TAA, PAJA, and the Constitution; taxpayer rights to just administrative action and court access; and appeal/objection rules.</t>
+  </si>
+  <si>
+    <t>Critically understand the concept of estate duty and its SA operation; understand the meaning of an "estate"; and explain components relevant to determining dutiable amounts.</t>
+  </si>
+  <si>
+    <t>Estate planning law.</t>
+  </si>
+  <si>
+    <t>Comprehend national/international dimensions of corruption; understand corruption as a barrier to development and human rights; and recognize/assess obstacles to anti-corruption practices.</t>
+  </si>
+  <si>
+    <t>Corruption meaning and extent; forms; evolution of law; SA anti-corruption statutes/cases; prevention and prosecution; collaboration; and asset recovery.</t>
+  </si>
+  <si>
+    <r>
+      <t>Consult the Criminal Justice and Procedure Department for detailed outcomes</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>Anti-money laundering law transnationally.</t>
+  </si>
+  <si>
+    <t>Apply comparative constitutional law methodology; and critically analyze constitutions regarding organizing government, rights models, constitutional review, and reform mechanisms.</t>
+  </si>
+  <si>
+    <t>Comparative law methodologies; principles; constitution making; systems/forms of government; judicial appointment; emergency powers; and review models.</t>
+  </si>
+  <si>
+    <t>Evaluate how a divided society's constitution can design state institutions to manage communities; demonstrate knowledge of constitutional choices for multi-ethnic states; and analyze options for polarized societies.</t>
+  </si>
+  <si>
+    <t>Challenges of divided societies; Bill of Rights response; constitutionalism; federalism; territorial pluralism; electoral systems; and language policy.</t>
+  </si>
+  <si>
+    <t>Analyze challenges facing rights interpretation in young democracies; understand hermeneutic/political factors; and identify and solve problems relating to specific constitutional rights.</t>
+  </si>
+  <si>
+    <t>Theories of interpretation; doctrines (separation of powers, popular constitutionalism); hermeneutic factors (text, values); and alternative theories (textualism, deconstruction).</t>
+  </si>
+  <si>
+    <t>Critically evaluate the concepts and ideas central to modern constitutions; and provide in-depth research analysis of covered topics.</t>
+  </si>
+  <si>
+    <t>The concept of the ‘political’ and the ‘constitution’; sovereignty; constituent power; democracy; and contemporary problems (e.g., right to the city, decolonial perspectives).</t>
+  </si>
+  <si>
+    <t>Acquire an understanding of how constitutional law is applied in practice; provide legal advice/opinions on interpretation in practical situations; and solve problems using creative thinking.</t>
+  </si>
+  <si>
+    <t>Practical research in constitutional law; internship experience at an institution of democracy; and praxis of application.</t>
+  </si>
+  <si>
+    <t>Analyze fundamental concepts and principles of constitutional interpretation in criminal justice; demonstrate knowledge of the Bill of Rights; and evaluate case law.</t>
+  </si>
+  <si>
+    <t>Bill of Rights examining: privacy and police powers (search/seizure); arrest and force; detainee rights (legal services); bail; and fair trial.</t>
+  </si>
+  <si>
+    <t>Analyze fundamental legal concepts, theories, and practices of intergovernmental relations in SA; and identify and solve problems regarding dispersal of powers and supervisory reach.</t>
+  </si>
+  <si>
+    <t>Multi-level governance.</t>
+  </si>
+  <si>
+    <t>Critically evaluate, apply, and reflect on concepts and theories relating to substantive gender equality and women’s rights; and conduct analysis from a gender perspective.</t>
+  </si>
+  <si>
+    <t>Gender equality and women’s rights.</t>
+  </si>
+  <si>
+    <t>Demonstrate knowledge of pluralism theories; challenge mainstream conceptualizations of customary law; explain pluralism as a product of legal history; and critique the indigenous-state law relationship.</t>
+  </si>
+  <si>
+    <t>Historical context; impact of colonial rule; major theories vs cultural relativism; customary law critique; dialogue areas between state and indigenous laws; and decolonization.</t>
+  </si>
+  <si>
+    <t>Children’s rights.</t>
+  </si>
+  <si>
+    <r>
+      <t>Consult the Global Environmental Law Centre for detailed outcomes</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>Climate change law and relevant governance; sectoral legislation; principles; international/SA actors; climate justice; and damages/liability.</t>
+  </si>
+  <si>
+    <t>Evaluate law for protecting nature and non-human animals; analyze taxonomy of environmental constitutionalism; and understand Earth Jurisprudence/non-anthropocentric approaches.</t>
+  </si>
+  <si>
+    <t>Governance scope for environment/nature; right holders; substantive/procedural rights; and concepts (Anthropocentrism, Rule of Law, Public Trust, Rights of Nature).</t>
+  </si>
+  <si>
+    <t>Critically evaluate the philosophical, ethical, scientific, and legal foundations of the protection of animals in South Africa and globally.</t>
+  </si>
+  <si>
+    <t>Current legal system deficiencies; core concepts (welfare, legal personhood, sentience, speciesism); and animal rights in the courts.</t>
+  </si>
+  <si>
+    <t>Analyze fundamental concepts and principles of corporate governance; examine main role players; evaluate SA regulation vs international practice; and identify shortcomings/solutions.</t>
+  </si>
+  <si>
+    <t>Theories of governance; King Reports (I-IV); role players; comparative studies (CSR, Ethical Leadership, Criminal Liability); and corporate law remedies.</t>
+  </si>
+  <si>
+    <t>Conceptualize Approach to financial regulation (Companies Act 2008); interpret decision-making principles for corporate finance; and explain rules for market abuse prevention.</t>
+  </si>
+  <si>
+    <t>SA/international principles; funding sources (equity); capital regulation (solvency/liquidity); distributions; and policy objectives of securities/financial markets.</t>
+  </si>
+  <si>
+    <t>Analyze options when a company enters the zone of insolvency; explain business rescue regulation and practice; and interpret relevant case law and statutes.</t>
+  </si>
+  <si>
+    <t>Corporate solvency principles; restructuring; business rescue framework (Practitioner powers, plan, termination); liquidations; and cross-border issues.</t>
+  </si>
+  <si>
+    <t>Demonstrate specialist knowledge of "property" (section 25); interpret regulatory control (planning, mining, neighbor law); and design alternative land reform strategies.</t>
+  </si>
+  <si>
+    <t>SA Bill of Rights (property); legal framework for regulatory control; methodological approaches; and the property relationship with other constitutional rights.</t>
+  </si>
+  <si>
+    <r>
+      <t>Consult the Private Law Department for detailed outcomes</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>Land reform and housing law.</t>
+  </si>
+  <si>
+    <t>Demonstrate specialist knowledge of competition theoretical underpinnings; explain competition economics; apply rules to practical scenarios; and analyze social justice relations.</t>
+  </si>
+  <si>
+    <t>Harvard/Chicago schools; economics/structures; horizontal/vertical practices; mergers; abuse of dominance; jurisdictions; and relations with IP, information, and labour law.</t>
+  </si>
+  <si>
+    <t>Identify and critically analyze the link between competition and labour law; analyze effects of employer monopsony power; and conceptualize "platform work" impact.</t>
+  </si>
+  <si>
+    <t>General principles/economics; market structures (monopsonies); defining workers; labour rights; Competition Act scope; and transformation/digitisation.</t>
+  </si>
+  <si>
+    <t>Conceptualize amalgamations/mergers and underpinning policies; interpret the legal framework (Companies Act 2008, Competition Act 1998); and explain takeover regulation.</t>
+  </si>
+  <si>
+    <t>Fundamental transactions; merger structures and effect; statutory merger procedures (Companies/Competition Acts); stakeholder protection; and the Takeover Regulation Panel.</t>
+  </si>
+  <si>
+    <t>Understand dynamic functions of a modern economy; conceptualize key areas of information law in the digital age; and critically evaluate competition in the digital economy.</t>
+  </si>
+  <si>
+    <t>Online consumer protection; privacy; computer crime; trade in digital services; AI; digital taxation; and technological approaches to enforcement in digital markets.</t>
+  </si>
+  <si>
+    <t>Demonstrate a specialist knowledge of the international legal framework relating to disability and the workplace.</t>
+  </si>
+  <si>
+    <t>Disability law and the workplace.</t>
+  </si>
+  <si>
+    <t>Negotiation, mediation, and arbitration processes; SA Truth and Reconciliation Commission; and restorative justice.</t>
+  </si>
+  <si>
+    <t>Demonstrate an understanding of, and ability to analyse, fundamental legal concepts of social protection.</t>
+  </si>
+  <si>
+    <t>The extension of social protection.</t>
+  </si>
+  <si>
+    <r>
+      <t>Consult the Centre for Legal Integration in Africa (CLIA) for detailed outcomes</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>International family law.</t>
+  </si>
+  <si>
+    <t>Appreciate the significance of corruption as an international crisis; understand it as a barrier to socio-economic development; and recognize obstacles to anti-corruption practices.</t>
+  </si>
+  <si>
+    <t>International anti-corruption law.</t>
+  </si>
+  <si>
+    <t>Evaluate what constitutes the "environment" internationally; and understand the application of international/regional policies and legal norms in SA domestic law.</t>
+  </si>
+  <si>
+    <t>IEL and SADC law pertaining to environment (SA perspective); Biodiversity; Sea/Wildlife law; Climate Change; and trade/development.</t>
+  </si>
+  <si>
+    <t>Critically evaluate the "environment"; identify ethical duties; identify complex environmentally related matters; and apply specialist knowledge to address/solve them.</t>
+  </si>
+  <si>
+    <t>Environment law scope; international/human rights dimensions; administration; implementation/enforcement; and natural/cultural resource utilization.</t>
+  </si>
+  <si>
+    <t>Demonstrate knowledge of international crimes; identify principles from sources to solve cases; evaluate ICC enforcement; and assess African reform/decolonisation proposals.</t>
+  </si>
+  <si>
+    <t>International criminal law.</t>
+  </si>
+  <si>
+    <t>Demonstrate knowledge of meaning/origin/debates; critically analyze AU approach within decolonized context; and conduct research for transitional justice scenarios.</t>
+  </si>
+  <si>
+    <t>Research/writing; theories (amnesty, truth, commissions); international law (Human rights/humanitarian); context studies (SA, Rwanda, DRC, etc.).</t>
+  </si>
+  <si>
+    <t>Comparative regional integration; trade; and human rights protection.</t>
+  </si>
+  <si>
+    <t>Demonstrate an understanding of fundamental concepts/principles/theories; and apply research methods and strategies to theoretical and applied situations.</t>
+  </si>
+  <si>
+    <t>Introduction to African, European, Inter-American, Asian, and Arab systems for human rights protection.</t>
+  </si>
+  <si>
+    <r>
+      <t>Consult the African Centre for Transnational Criminal Justice for detailed outcomes</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <t>International humanitarian law.</t>
+  </si>
+  <si>
+    <t>Critically analyze contemporary human rights issues; evaluate monitoring limits and politicization; and analyze links between rights, development, and poverty.</t>
+  </si>
+  <si>
+    <t>Global human rights issues.</t>
+  </si>
+  <si>
+    <t>Critically discuss fundamental legal theories, concepts, and principles of intellectual property.</t>
+  </si>
+  <si>
+    <t>Intellectual property law.</t>
+  </si>
+  <si>
+    <t>Demonstrate an understanding of concepts and principles; and apply methods and strategies involved in legal research and problem solving.</t>
+  </si>
+  <si>
+    <t>International trade law practices; international economic/trade dispute settlement (arbitration).</t>
+  </si>
+  <si>
+    <t>Demonstrate an understanding of concepts, principles, theories, and their relationship to international business practices.</t>
+  </si>
+  <si>
+    <t>Sales, finance, and competition forms; arbitration; environmental/social considerations; EU Law; AGOA, SADC, AU roles; and African trade negotiation roles.</t>
+  </si>
+  <si>
+    <t>Demonstrate an understanding of, and ability to analyse, fundamental legal concepts and principles of investment law.</t>
+  </si>
+  <si>
+    <t>Public/private international law; state responsibility; treaties; global institutes (UNCTAD, AfDB, IMF); WTO regulation; IP (TRIPS); and investment regulation in Africa.</t>
+  </si>
+  <si>
+    <t>Critically analyze concepts/theories of international taxation; evaluate OECD models vs SA; interpret rules for double tax agreements; and argue for decolonized principles.</t>
+  </si>
+  <si>
+    <t>Jurisdiction (source/residence); treatment of income for different taxpayers; international headquarter companies; double tax agreements; and Constitution impact.</t>
+  </si>
+  <si>
+    <t>Collective bargaining and minimum standards in non-standard employment markets; workplace equality/affirmative action; and 4IR context.</t>
+  </si>
+  <si>
+    <t>Analyze concepts, principles, and theories relevant to dismissal development; and apply research methods and strategies.</t>
+  </si>
+  <si>
+    <t>Law of unfair dismissal.</t>
+  </si>
+  <si>
+    <t>Demonstrate understanding of rule of law principles; critically discuss SA constitutionalism; evaluate SA system in international debates; and critically analyze/solve problems.</t>
+  </si>
+  <si>
+    <t>Constitutional governance; rule of law; internal/external accountability; Chapter 9 institutions; PAIA; procurement; PAJA; review; Ubuntu; and digital impact.</t>
+  </si>
+  <si>
+    <t>Demonstrate an understanding of, and ability to analyse, fundamental legal concepts, principles, theories, and practices of local government in SA.</t>
+  </si>
+  <si>
+    <t>Penalty clauses in international treaties; minimum/mandatory sentences; judicial discretion; mitigation/aggravation; and Bill of Rights relationship.</t>
+  </si>
+  <si>
+    <t>Demonstrate an understanding of how the crime of money laundering developed transnationally.</t>
+  </si>
+  <si>
+    <t>International anti-money laundering law.</t>
+  </si>
+  <si>
+    <t>Critically analyze schools of religious thought in Islam; assess conflict between rights approaches and scriptural interpretation; and evaluate state/non-state roles.</t>
+  </si>
+  <si>
+    <t>Muslim Personal Law.</t>
+  </si>
+  <si>
+    <t>Understand theories relating to enforcement; apply research methods; identify international instruments/oversight bodies; and engage with separation of powers issues.</t>
+  </si>
+  <si>
+    <t>Economic, social, and cultural rights.</t>
+  </si>
+  <si>
+    <t>Demonstrate understanding of trade/investment/business transactions; evaluate conflicts; analyze settlement legitimacy based on jurisprudence; and formulate views on shortcomings.</t>
+  </si>
+  <si>
+    <t>Dispute settlement in international transactions.</t>
+  </si>
+  <si>
+    <t>Analyze rules under the TAA, PAJA, and the Constitution; explain taxpayer rights (privacy, property, access); and interpret rules for appeals and objections.</t>
+  </si>
+  <si>
+    <t>Provisions of TAA, PAJA, and the Constitution; inter-relationships; taxpayer rights; and court/tribunal access.</t>
+  </si>
+  <si>
+    <t>Made a satisfactory contribution to knowledge in Law or its interaction with another discipline by either proposing a significant research question or through substantial studies.</t>
+  </si>
+  <si>
+    <t>Research project in any area of Law or interaction with another field.</t>
+  </si>
+  <si>
+    <t>Made a limited scope contribution to knowledge in Law or interaction with another discipline following a research question with potential.</t>
+  </si>
+  <si>
+    <t>Research proposals from any area of Law; interaction with another field; and substantial historical or comparative studies.</t>
+  </si>
+  <si>
+    <t>Made a limited scope contribution to knowledge in Law following a research question with satisfactory potential; carry out and report on research.</t>
+  </si>
+  <si>
+    <t>Mini-thesis in Legal Pluralism and Family Law.</t>
+  </si>
+  <si>
+    <t>Made a limited scope contribution to knowledge in Law; carry out and report on research in an approximately 18,000-word paper suitable for publication.</t>
+  </si>
+  <si>
+    <t>Research Paper.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -569,6 +1121,14 @@
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -596,7 +1156,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -605,6 +1165,9 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -622,6 +1185,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -887,13 +1454,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F79"/>
+  <dimension ref="A1:I79"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="4" max="4" width="26.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -912,8 +1479,17 @@
       <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="G1" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
@@ -932,8 +1508,17 @@
       <c r="F2" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="3" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="G2" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="I2" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>9</v>
       </c>
@@ -952,8 +1537,17 @@
       <c r="F3" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="4" spans="1:6" ht="115.2" x14ac:dyDescent="0.3">
+      <c r="G3" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="I3" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="403.2" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>11</v>
       </c>
@@ -972,8 +1566,17 @@
       <c r="F4" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="G4" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="I4" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="201.6" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>13</v>
       </c>
@@ -992,8 +1595,17 @@
       <c r="F5" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="6" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="G5" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="I5" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="388.8" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>15</v>
       </c>
@@ -1012,8 +1624,17 @@
       <c r="F6" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="7" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="G6" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="I6" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="331.2" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>17</v>
       </c>
@@ -1032,8 +1653,17 @@
       <c r="F7" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="8" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="G7" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="I7" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="388.8" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>19</v>
       </c>
@@ -1052,8 +1682,17 @@
       <c r="F8" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="9" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="G8" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="I8" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="201.6" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>21</v>
       </c>
@@ -1072,8 +1711,17 @@
       <c r="F9" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" ht="72" x14ac:dyDescent="0.3">
+      <c r="G9" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="I9" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="244.8" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>23</v>
       </c>
@@ -1092,8 +1740,17 @@
       <c r="F10" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" ht="72" x14ac:dyDescent="0.3">
+      <c r="G10" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="I10" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="288" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>25</v>
       </c>
@@ -1112,8 +1769,17 @@
       <c r="F11" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" ht="72" x14ac:dyDescent="0.3">
+      <c r="G11" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="I11" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>27</v>
       </c>
@@ -1132,8 +1798,17 @@
       <c r="F12" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="G12" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="I12" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="360" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>29</v>
       </c>
@@ -1152,8 +1827,17 @@
       <c r="F13" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="G13" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="I13" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="360" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>31</v>
       </c>
@@ -1172,8 +1856,17 @@
       <c r="F14" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="G14" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="I14" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="360" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>33</v>
       </c>
@@ -1192,8 +1885,17 @@
       <c r="F15" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="16" spans="1:6" ht="72" x14ac:dyDescent="0.3">
+      <c r="G15" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="H15" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="I15" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="374.4" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>35</v>
       </c>
@@ -1212,8 +1914,17 @@
       <c r="F16" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="17" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="G16" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="H16" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="I16" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>37</v>
       </c>
@@ -1232,8 +1943,17 @@
       <c r="F17" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="18" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="G17" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="H17" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="I17" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="316.8" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>39</v>
       </c>
@@ -1252,8 +1972,17 @@
       <c r="F18" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="19" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="G18" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="H18" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="I18" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" ht="216" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>41</v>
       </c>
@@ -1272,8 +2001,17 @@
       <c r="F19" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="G19" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="H19" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="I19" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" ht="360" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
         <v>43</v>
       </c>
@@ -1292,8 +2030,17 @@
       <c r="F20" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="G20" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="H20" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="I20" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" ht="345.6" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
         <v>45</v>
       </c>
@@ -1312,8 +2059,17 @@
       <c r="F21" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="22" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="G21" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="H21" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="I21" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" ht="331.2" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>47</v>
       </c>
@@ -1332,8 +2088,17 @@
       <c r="F22" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="23" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="G22" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="H22" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="I22" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" ht="345.6" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
         <v>49</v>
       </c>
@@ -1352,8 +2117,17 @@
       <c r="F23" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="24" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="G23" s="1" t="s">
+        <v>220</v>
+      </c>
+      <c r="H23" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="I23" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" ht="374.4" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
         <v>51</v>
       </c>
@@ -1372,8 +2146,17 @@
       <c r="F24" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="25" spans="1:6" ht="72" x14ac:dyDescent="0.3">
+      <c r="G24" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="H24" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="I24" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" ht="172.8" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
         <v>53</v>
       </c>
@@ -1392,8 +2175,17 @@
       <c r="F25" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="26" spans="1:6" ht="72" x14ac:dyDescent="0.3">
+      <c r="G25" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="H25" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="I25" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" ht="360" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
         <v>55</v>
       </c>
@@ -1412,8 +2204,17 @@
       <c r="F26" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="27" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="G26" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="H26" s="1" t="s">
+        <v>227</v>
+      </c>
+      <c r="I26" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
         <v>57</v>
       </c>
@@ -1432,8 +2233,17 @@
       <c r="F27" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="28" spans="1:6" ht="72" x14ac:dyDescent="0.3">
+      <c r="G27" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="H27" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="I27" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" ht="360" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
         <v>59</v>
       </c>
@@ -1452,8 +2262,17 @@
       <c r="F28" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="29" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="G28" s="1" t="s">
+        <v>230</v>
+      </c>
+      <c r="H28" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="I28" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" ht="331.2" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
         <v>61</v>
       </c>
@@ -1472,8 +2291,17 @@
       <c r="F29" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="30" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="G29" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="H29" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="I29" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" ht="360" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>63</v>
       </c>
@@ -1492,8 +2320,17 @@
       <c r="F30" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="31" spans="1:6" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="G30" s="1" t="s">
+        <v>234</v>
+      </c>
+      <c r="H30" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="I30" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" ht="316.8" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
         <v>65</v>
       </c>
@@ -1512,8 +2349,17 @@
       <c r="F31" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="32" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="G31" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="H31" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="I31" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" ht="316.8" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
         <v>67</v>
       </c>
@@ -1532,8 +2378,17 @@
       <c r="F32" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="33" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="G32" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="H32" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="I32" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" ht="331.2" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
         <v>69</v>
       </c>
@@ -1552,8 +2407,17 @@
       <c r="F33" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="34" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="G33" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="H33" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="I33" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" ht="403.2" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
         <v>71</v>
       </c>
@@ -1572,8 +2436,17 @@
       <c r="F34" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="35" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="G34" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="H34" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="I34" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
         <v>73</v>
       </c>
@@ -1592,8 +2465,17 @@
       <c r="F35" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="36" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="G35" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="H35" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="I35" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" ht="273.60000000000002" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
         <v>75</v>
       </c>
@@ -1612,8 +2494,17 @@
       <c r="F36" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="37" spans="1:6" ht="72" x14ac:dyDescent="0.3">
+      <c r="G36" s="4" t="s">
+        <v>245</v>
+      </c>
+      <c r="H36" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="I36" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" ht="331.2" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
         <v>78</v>
       </c>
@@ -1632,8 +2523,17 @@
       <c r="F37" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="38" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="G37" s="1" t="s">
+        <v>247</v>
+      </c>
+      <c r="H37" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="I37" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" ht="259.2" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
         <v>80</v>
       </c>
@@ -1652,8 +2552,17 @@
       <c r="F38" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="39" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="G38" s="1" t="s">
+        <v>249</v>
+      </c>
+      <c r="H38" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="I38" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" ht="374.4" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
         <v>82</v>
       </c>
@@ -1672,8 +2581,17 @@
       <c r="F39" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="40" spans="1:6" ht="72" x14ac:dyDescent="0.3">
+      <c r="G39" s="1" t="s">
+        <v>251</v>
+      </c>
+      <c r="H39" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="I39" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" ht="360" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
         <v>84</v>
       </c>
@@ -1692,8 +2610,17 @@
       <c r="F40" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="41" spans="1:6" ht="72" x14ac:dyDescent="0.3">
+      <c r="G40" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="H40" s="1" t="s">
+        <v>254</v>
+      </c>
+      <c r="I40" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" ht="316.8" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
         <v>86</v>
       </c>
@@ -1712,8 +2639,17 @@
       <c r="F41" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="42" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="G41" s="1" t="s">
+        <v>255</v>
+      </c>
+      <c r="H41" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="I41" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" ht="302.39999999999998" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
         <v>88</v>
       </c>
@@ -1732,8 +2668,17 @@
       <c r="F42" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="43" spans="1:6" ht="72" x14ac:dyDescent="0.3">
+      <c r="G42" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="H42" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="I42" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
         <v>90</v>
       </c>
@@ -1752,8 +2697,17 @@
       <c r="F43" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="44" spans="1:6" ht="72" x14ac:dyDescent="0.3">
+      <c r="G43" s="4" t="s">
+        <v>259</v>
+      </c>
+      <c r="H43" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="I43" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" ht="345.6" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
         <v>92</v>
       </c>
@@ -1772,8 +2726,17 @@
       <c r="F44" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="45" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="G44" s="1" t="s">
+        <v>261</v>
+      </c>
+      <c r="H44" s="1" t="s">
+        <v>262</v>
+      </c>
+      <c r="I44" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" ht="316.8" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
         <v>94</v>
       </c>
@@ -1792,8 +2755,17 @@
       <c r="F45" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="46" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="G45" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="H45" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="I45" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" ht="345.6" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
         <v>96</v>
       </c>
@@ -1812,8 +2784,17 @@
       <c r="F46" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="47" spans="1:6" ht="72" x14ac:dyDescent="0.3">
+      <c r="G46" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="H46" s="1" t="s">
+        <v>266</v>
+      </c>
+      <c r="I46" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" ht="331.2" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
         <v>98</v>
       </c>
@@ -1832,8 +2813,17 @@
       <c r="F47" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="48" spans="1:6" ht="72" x14ac:dyDescent="0.3">
+      <c r="G47" s="1" t="s">
+        <v>267</v>
+      </c>
+      <c r="H47" s="1" t="s">
+        <v>268</v>
+      </c>
+      <c r="I47" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" ht="216" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
         <v>100</v>
       </c>
@@ -1852,8 +2842,17 @@
       <c r="F48" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="49" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="G48" s="1" t="s">
+        <v>269</v>
+      </c>
+      <c r="H48" s="1" t="s">
+        <v>270</v>
+      </c>
+      <c r="I48" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" ht="216" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
         <v>102</v>
       </c>
@@ -1872,8 +2871,17 @@
       <c r="F49" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="50" spans="1:6" ht="72" x14ac:dyDescent="0.3">
+      <c r="G49" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="H49" s="1" t="s">
+        <v>271</v>
+      </c>
+      <c r="I49" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
         <v>104</v>
       </c>
@@ -1892,8 +2900,17 @@
       <c r="F50" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="51" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="G50" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="H50" s="1" t="s">
+        <v>273</v>
+      </c>
+      <c r="I50" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A51" s="2" t="s">
         <v>106</v>
       </c>
@@ -1912,8 +2929,17 @@
       <c r="F51" s="1" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="52" spans="1:6" ht="72" x14ac:dyDescent="0.3">
+      <c r="G51" s="4" t="s">
+        <v>274</v>
+      </c>
+      <c r="H51" s="1" t="s">
+        <v>275</v>
+      </c>
+      <c r="I51" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9" ht="345.6" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
         <v>108</v>
       </c>
@@ -1932,8 +2958,17 @@
       <c r="F52" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="53" spans="1:6" ht="72" x14ac:dyDescent="0.3">
+      <c r="G52" s="1" t="s">
+        <v>276</v>
+      </c>
+      <c r="H52" s="1" t="s">
+        <v>277</v>
+      </c>
+      <c r="I52" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9" ht="316.8" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
         <v>110</v>
       </c>
@@ -1952,8 +2987,17 @@
       <c r="F53" s="1" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="54" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="G53" s="1" t="s">
+        <v>278</v>
+      </c>
+      <c r="H53" s="1" t="s">
+        <v>279</v>
+      </c>
+      <c r="I53" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" ht="302.39999999999998" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
         <v>77</v>
       </c>
@@ -1972,8 +3016,17 @@
       <c r="F54" s="1" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="55" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="G54" s="1" t="s">
+        <v>280</v>
+      </c>
+      <c r="H54" s="1" t="s">
+        <v>281</v>
+      </c>
+      <c r="I54" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" ht="345.6" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
         <v>115</v>
       </c>
@@ -1992,8 +3045,17 @@
       <c r="F55" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="56" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="G55" s="1" t="s">
+        <v>282</v>
+      </c>
+      <c r="H55" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="I55" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" ht="331.2" x14ac:dyDescent="0.3">
       <c r="A56" s="2" t="s">
         <v>117</v>
       </c>
@@ -2012,8 +3074,17 @@
       <c r="F56" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="57" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="G56" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="H56" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="I56" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A57" s="2" t="s">
         <v>119</v>
       </c>
@@ -2032,8 +3103,17 @@
       <c r="F57" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="58" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="G57" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="H57" s="1" t="s">
+        <v>286</v>
+      </c>
+      <c r="I57" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" ht="302.39999999999998" x14ac:dyDescent="0.3">
       <c r="A58" s="2" t="s">
         <v>121</v>
       </c>
@@ -2052,8 +3132,17 @@
       <c r="F58" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="59" spans="1:6" ht="72" x14ac:dyDescent="0.3">
+      <c r="G58" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="H58" s="1" t="s">
+        <v>288</v>
+      </c>
+      <c r="I58" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A59" s="2" t="s">
         <v>123</v>
       </c>
@@ -2072,8 +3161,17 @@
       <c r="F59" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="60" spans="1:6" ht="72" x14ac:dyDescent="0.3">
+      <c r="G59" s="4" t="s">
+        <v>289</v>
+      </c>
+      <c r="H59" s="1" t="s">
+        <v>290</v>
+      </c>
+      <c r="I59" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" ht="302.39999999999998" x14ac:dyDescent="0.3">
       <c r="A60" s="2" t="s">
         <v>125</v>
       </c>
@@ -2092,8 +3190,17 @@
       <c r="F60" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="61" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="G60" s="1" t="s">
+        <v>291</v>
+      </c>
+      <c r="H60" s="1" t="s">
+        <v>292</v>
+      </c>
+      <c r="I60" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9" ht="172.8" x14ac:dyDescent="0.3">
       <c r="A61" s="2" t="s">
         <v>127</v>
       </c>
@@ -2112,8 +3219,17 @@
       <c r="F61" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="62" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="G61" s="1" t="s">
+        <v>293</v>
+      </c>
+      <c r="H61" s="1" t="s">
+        <v>294</v>
+      </c>
+      <c r="I61" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="62" spans="1:9" ht="259.2" x14ac:dyDescent="0.3">
       <c r="A62" s="2" t="s">
         <v>129</v>
       </c>
@@ -2132,8 +3248,17 @@
       <c r="F62" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="63" spans="1:6" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="G62" s="1" t="s">
+        <v>295</v>
+      </c>
+      <c r="H62" s="1" t="s">
+        <v>296</v>
+      </c>
+      <c r="I62" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="63" spans="1:9" ht="302.39999999999998" x14ac:dyDescent="0.3">
       <c r="A63" s="2" t="s">
         <v>131</v>
       </c>
@@ -2152,8 +3277,17 @@
       <c r="F63" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="64" spans="1:6" ht="100.8" x14ac:dyDescent="0.3">
+      <c r="G63" s="1" t="s">
+        <v>297</v>
+      </c>
+      <c r="H63" s="1" t="s">
+        <v>298</v>
+      </c>
+      <c r="I63" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="64" spans="1:9" ht="331.2" x14ac:dyDescent="0.3">
       <c r="A64" s="2" t="s">
         <v>133</v>
       </c>
@@ -2172,8 +3306,17 @@
       <c r="F64" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="65" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="G64" s="1" t="s">
+        <v>299</v>
+      </c>
+      <c r="H64" s="1" t="s">
+        <v>300</v>
+      </c>
+      <c r="I64" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="65" spans="1:9" ht="360" x14ac:dyDescent="0.3">
       <c r="A65" s="2" t="s">
         <v>135</v>
       </c>
@@ -2192,8 +3335,17 @@
       <c r="F65" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="66" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="G65" s="1" t="s">
+        <v>301</v>
+      </c>
+      <c r="H65" s="1" t="s">
+        <v>302</v>
+      </c>
+      <c r="I65" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="66" spans="1:9" ht="273.60000000000002" x14ac:dyDescent="0.3">
       <c r="A66" s="2" t="s">
         <v>137</v>
       </c>
@@ -2212,8 +3364,17 @@
       <c r="F66" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="67" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="G66" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="H66" s="1" t="s">
+        <v>303</v>
+      </c>
+      <c r="I66" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="67" spans="1:9" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A67" s="2" t="s">
         <v>139</v>
       </c>
@@ -2232,8 +3393,17 @@
       <c r="F67" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="68" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="G67" s="1" t="s">
+        <v>304</v>
+      </c>
+      <c r="H67" s="1" t="s">
+        <v>305</v>
+      </c>
+      <c r="I67" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="68" spans="1:9" ht="345.6" x14ac:dyDescent="0.3">
       <c r="A68" s="2" t="s">
         <v>141</v>
       </c>
@@ -2252,8 +3422,17 @@
       <c r="F68" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="69" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="G68" s="1" t="s">
+        <v>306</v>
+      </c>
+      <c r="H68" s="1" t="s">
+        <v>307</v>
+      </c>
+      <c r="I68" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="69" spans="1:9" ht="259.2" x14ac:dyDescent="0.3">
       <c r="A69" s="2" t="s">
         <v>143</v>
       </c>
@@ -2272,8 +3451,17 @@
       <c r="F69" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="70" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="G69" s="1" t="s">
+        <v>308</v>
+      </c>
+      <c r="H69" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="I69" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="70" spans="1:9" ht="273.60000000000002" x14ac:dyDescent="0.3">
       <c r="A70" s="2" t="s">
         <v>145</v>
       </c>
@@ -2292,8 +3480,17 @@
       <c r="F70" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="71" spans="1:6" ht="72" x14ac:dyDescent="0.3">
+      <c r="G70" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="H70" s="1" t="s">
+        <v>309</v>
+      </c>
+      <c r="I70" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="71" spans="1:9" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A71" s="2" t="s">
         <v>147</v>
       </c>
@@ -2312,8 +3509,17 @@
       <c r="F71" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="72" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="G71" s="1" t="s">
+        <v>310</v>
+      </c>
+      <c r="H71" s="1" t="s">
+        <v>311</v>
+      </c>
+      <c r="I71" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="72" spans="1:9" ht="302.39999999999998" x14ac:dyDescent="0.3">
       <c r="A72" s="2" t="s">
         <v>149</v>
       </c>
@@ -2332,8 +3538,17 @@
       <c r="F72" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="73" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="G72" s="1" t="s">
+        <v>312</v>
+      </c>
+      <c r="H72" s="1" t="s">
+        <v>313</v>
+      </c>
+      <c r="I72" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="73" spans="1:9" ht="345.6" x14ac:dyDescent="0.3">
       <c r="A73" s="2" t="s">
         <v>151</v>
       </c>
@@ -2352,8 +3567,17 @@
       <c r="F73" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="74" spans="1:6" ht="72" x14ac:dyDescent="0.3">
+      <c r="G73" s="1" t="s">
+        <v>314</v>
+      </c>
+      <c r="H73" s="1" t="s">
+        <v>315</v>
+      </c>
+      <c r="I73" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="74" spans="1:9" ht="345.6" x14ac:dyDescent="0.3">
       <c r="A74" s="2" t="s">
         <v>153</v>
       </c>
@@ -2372,8 +3596,17 @@
       <c r="F74" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="75" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="G74" s="1" t="s">
+        <v>316</v>
+      </c>
+      <c r="H74" s="1" t="s">
+        <v>317</v>
+      </c>
+      <c r="I74" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="75" spans="1:9" ht="302.39999999999998" x14ac:dyDescent="0.3">
       <c r="A75" s="2" t="s">
         <v>155</v>
       </c>
@@ -2392,8 +3625,17 @@
       <c r="F75" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="76" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="G75" s="1" t="s">
+        <v>318</v>
+      </c>
+      <c r="H75" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="I75" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="76" spans="1:9" ht="345.6" x14ac:dyDescent="0.3">
       <c r="A76" s="2" t="s">
         <v>157</v>
       </c>
@@ -2412,8 +3654,17 @@
       <c r="F76" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="77" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="G76" s="1" t="s">
+        <v>320</v>
+      </c>
+      <c r="H76" s="1" t="s">
+        <v>321</v>
+      </c>
+      <c r="I76" s="1">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="77" spans="1:9" ht="259.2" x14ac:dyDescent="0.3">
       <c r="A77" s="2" t="s">
         <v>159</v>
       </c>
@@ -2432,8 +3683,17 @@
       <c r="F77" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="78" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
+      <c r="G77" s="1" t="s">
+        <v>322</v>
+      </c>
+      <c r="H77" s="1" t="s">
+        <v>323</v>
+      </c>
+      <c r="I77" s="1">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="78" spans="1:9" ht="273.60000000000002" x14ac:dyDescent="0.3">
       <c r="A78" s="2" t="s">
         <v>161</v>
       </c>
@@ -2452,8 +3712,17 @@
       <c r="F78" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="79" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="G78" s="1" t="s">
+        <v>324</v>
+      </c>
+      <c r="H78" s="1" t="s">
+        <v>325</v>
+      </c>
+      <c r="I78" s="1">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="79" spans="1:9" ht="302.39999999999998" x14ac:dyDescent="0.3">
       <c r="A79" s="2" t="s">
         <v>163</v>
       </c>
@@ -2471,6 +3740,15 @@
       </c>
       <c r="F79" s="1" t="s">
         <v>8</v>
+      </c>
+      <c r="G79" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="H79" s="1" t="s">
+        <v>327</v>
+      </c>
+      <c r="I79" s="1">
+        <v>60</v>
       </c>
     </row>
   </sheetData>

</xml_diff>